<commit_message>
Complete Stage 2 audit: final workbook, findings, README, prompt log
Swapped in the fully audited model.xlsx (Solver run twice from different
starting points, both converging on 10 tomato / 20 carrot / 30 mesclun
beds at $42,775.17 profit; Farm Profit Lab cross-check within $0.89;
zero formula errors across 788 formulas).

Appended 5 audit findings to spec.md: the two Solver runs agreeing, the
Farm Profit Lab match, the crossing-point defect found and fixed, a GRG
Nonlinear precision residue on TOM_BEDS (10.0045 vs. exactly 10), and the
$13 season-profit gap traced to the case's own CAR_HRS = 0.833 input
precision rather than a formula defect.

Updated README.md with the capability description and an "exercised in"
link to the Perfect Competition brief, and logged this session in
prompt-log.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gm6T67PcpZgDaTHre5FcNB
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" state="visible" r:id="rId3"/>
@@ -69,6 +69,50 @@
     <definedName function="false" hidden="false" name="WEEKS" vbProcedure="false">Inputs!$B$19</definedName>
     <definedName function="false" hidden="false" name="WORKER_HRS" vbProcedure="false">Inputs!$B$25</definedName>
     <definedName function="false" hidden="false" name="WORKER_RATE" vbProcedure="false">Inputs!$B$26</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_adj" vbProcedure="false">Optimization!$B$4:$B$6</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_cvg" vbProcedure="false">0.0000001</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_drv" vbProcedure="false">1</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_eng" vbProcedure="false">1</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_itr" vbProcedure="false">2147483647</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_lhs1" vbProcedure="false">Optimization!$B$36</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_lhs2" vbProcedure="false">Optimization!$B$38</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_lhs3" vbProcedure="false">Optimization!$B$4:$B$6</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_lhs4" vbProcedure="false">Optimization!$B$5</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_lhs5" vbProcedure="false">Optimization!$B$6</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_lhs6" vbProcedure="false">Optimization!$B$4</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_lin" vbProcedure="false">2</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_mip" vbProcedure="false">2147483647</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_mni" vbProcedure="false">30</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_mrt" vbProcedure="false">0.075</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_msl" vbProcedure="false">2</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_neg" vbProcedure="false">1</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_nod" vbProcedure="false">2147483647</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_num" vbProcedure="false">6</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_opt" vbProcedure="false">Optimization!$B$22</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_pre" vbProcedure="false">0.000001</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_rbv" vbProcedure="false">1</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_rel1" vbProcedure="false">1</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_rel2" vbProcedure="false">1</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_rel3" vbProcedure="false">4</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_rel4" vbProcedure="false">1</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_rel5" vbProcedure="false">1</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_rel6" vbProcedure="false">1</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_rhs1" vbProcedure="false">Optimization!$B$35</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_rhs2" vbProcedure="false">Optimization!$B$37</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_rhs3" vbProcedure="false">"integer"</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_rhs4" vbProcedure="false">Optimization!$B$33</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_rhs5" vbProcedure="false">Optimization!$B$34</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_rhs6" vbProcedure="false">Optimization!$B$32</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_rlx" vbProcedure="false">1</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_rsd" vbProcedure="false">0</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_scl" vbProcedure="false">2</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_sho" vbProcedure="false">2</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_ssz" vbProcedure="false">100</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_tim" vbProcedure="false">2147483647</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_tol" vbProcedure="false">0</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_typ" vbProcedure="false">1</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_val" vbProcedure="false">0</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="solver_ver" vbProcedure="false">2</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -80,7 +124,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="152">
   <si>
     <t xml:space="preserve">Inputs</t>
   </si>
@@ -275,6 +319,27 @@
   </si>
   <si>
     <t xml:space="preserve">TOM_BEDS, CAR_BEDS, MES_BEDS must be set to 'int' (integer) in Solver constraints</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tomato Cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carrot Cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mesclun Cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Beds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Beds Planted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max Temp Labor Hours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Temp Hours Used (link)</t>
   </si>
   <si>
     <t xml:space="preserve">Cost Structure</t>
@@ -556,7 +621,7 @@
       <b val="true"/>
       <sz val="14"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
@@ -564,35 +629,35 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="11"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="12"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -656,7 +721,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -713,6 +778,18 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -754,7 +831,87 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="10">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -1020,7 +1177,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D26"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
@@ -1385,8 +1542,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:B38"/>
+  <sheetFormatPr defaultColWidth="8.5" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
@@ -1407,7 +1564,7 @@
         <v>42</v>
       </c>
       <c r="B4" s="10" t="n">
-        <v>0</v>
+        <v>10.004470073479</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1415,7 +1572,7 @@
         <v>43</v>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1423,7 +1580,7 @@
         <v>44</v>
       </c>
       <c r="B6" s="10" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1437,7 +1594,7 @@
       </c>
       <c r="B9" s="11" t="n">
         <f aca="false">TOM_BEDS*TOM_PRICE</f>
-        <v>0</v>
+        <v>88039.3366466152</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1446,7 +1603,7 @@
       </c>
       <c r="B10" s="11" t="n">
         <f aca="false">CAR_BEDS*CAR_PRICE</f>
-        <v>0</v>
+        <v>41880</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1455,7 +1612,7 @@
       </c>
       <c r="B11" s="11" t="n">
         <f aca="false">MES_BEDS*MES_PRICE</f>
-        <v>0</v>
+        <v>81000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1464,7 +1621,7 @@
       </c>
       <c r="B12" s="12" t="n">
         <f aca="false">SUM(B9:B11)</f>
-        <v>0</v>
+        <v>210919.336646615</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1478,7 +1635,7 @@
       </c>
       <c r="B15" s="11" t="n">
         <f aca="false">TOTAL_LABOR_DOLLARS</f>
-        <v>0</v>
+        <v>104140.236074781</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1487,7 +1644,7 @@
       </c>
       <c r="B16" s="11" t="n">
         <f aca="false">TOTAL_FERT_COST</f>
-        <v>0</v>
+        <v>44003.9336646615</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1496,7 +1653,7 @@
       </c>
       <c r="B17" s="11" t="n">
         <f aca="false">B15+B16</f>
-        <v>0</v>
+        <v>148144.169739442</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1514,7 +1671,7 @@
       </c>
       <c r="B19" s="12" t="n">
         <f aca="false">B17+B18</f>
-        <v>20000</v>
+        <v>168144.169739442</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1528,7 +1685,7 @@
       </c>
       <c r="B22" s="13" t="n">
         <f aca="false">TOTAL_REVENUE-TOTAL_COST</f>
-        <v>-20000</v>
+        <v>42775.1669071729</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1564,6 +1721,69 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
         <v>64</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B32" s="14" t="n">
+        <f aca="false">TOM_CAP</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B33" s="14" t="n">
+        <f aca="false">CAR_CAP</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B34" s="14" t="n">
+        <f aca="false">MES_CAP</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B35" s="14" t="n">
+        <f aca="false">TOTAL_BEDS</f>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B36" s="15" t="n">
+        <f aca="false">TOM_BEDS+CAR_BEDS+MES_BEDS</f>
+        <v>60.004470073479</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B37" s="15" t="n">
+        <f aca="false">MAX_WORKERS*WORKER_HRS</f>
+        <v>5760</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B38" s="16" t="n">
+        <f aca="false">'Cost Structure'!B8</f>
+        <v>4558.86152504498</v>
       </c>
     </row>
   </sheetData>
@@ -1583,7 +1803,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="16"/>
@@ -1591,119 +1811,119 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B4" s="14" t="n">
+        <v>78</v>
+      </c>
+      <c r="B4" s="17" t="n">
         <f aca="false">TOM_BEDS*TOM_HRS*WEEKS*(1+TOM_DIM)^TOM_BEDS</f>
-        <v>0</v>
-      </c>
-      <c r="C4" s="14" t="n">
+        <v>2336.40689280676</v>
+      </c>
+      <c r="C4" s="17" t="n">
         <f aca="false">CAR_BEDS*CAR_HRS*WEEKS*(1+CAR_DIM)^CAR_BEDS</f>
-        <v>0</v>
-      </c>
-      <c r="D4" s="14" t="n">
+        <v>982.776596228567</v>
+      </c>
+      <c r="D4" s="17" t="n">
         <f aca="false">MES_BEDS*MES_HRS*WEEKS*(1+MES_DIM)^MES_BEDS</f>
-        <v>0</v>
-      </c>
-      <c r="E4" s="15" t="n">
+        <v>1959.67803600965</v>
+      </c>
+      <c r="E4" s="18" t="n">
         <f aca="false">SUM(B4:D4)</f>
-        <v>0</v>
+        <v>5278.86152504498</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="B5" s="11" t="n">
         <f aca="false">TOM_BEDS*TOM_FERT</f>
-        <v>0</v>
+        <v>8803.93366466152</v>
       </c>
       <c r="C5" s="11" t="n">
         <f aca="false">CAR_BEDS*CAR_FERT</f>
-        <v>0</v>
+        <v>8800</v>
       </c>
       <c r="D5" s="11" t="n">
         <f aca="false">MES_BEDS*MES_FERT</f>
-        <v>0</v>
+        <v>26400</v>
       </c>
       <c r="E5" s="12" t="n">
         <f aca="false">SUM(B5:D5)</f>
-        <v>0</v>
+        <v>44003.9336646615</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B7" s="14" t="n">
+        <v>80</v>
+      </c>
+      <c r="B7" s="17" t="n">
         <f aca="false">MIN(TOTAL_HRS,OWN_HRS)</f>
-        <v>0</v>
+        <v>720</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="B8" s="14" t="n">
+        <v>81</v>
+      </c>
+      <c r="B8" s="17" t="n">
         <f aca="false">MAX(TOTAL_HRS-OWN_HRS,0)</f>
-        <v>0</v>
+        <v>4558.86152504498</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B9" s="12" t="n">
         <f aca="false">FARMER_HRS_USED*OWN_RATE+TEMP_HRS_USED*WORKER_RATE</f>
-        <v>0</v>
+        <v>104140.236074781</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="B10" s="12" t="n">
         <f aca="false">IF(TOTAL_HRS=0,0,TOTAL_LABOR_DOLLARS/TOTAL_HRS)</f>
-        <v>0</v>
+        <v>19.7277832693089</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="B12" s="11" t="n">
         <f aca="false">LABOR_HRS_TOM*BLENDED_RATE</f>
-        <v>0</v>
+        <v>46092.1288102113</v>
       </c>
       <c r="C12" s="11" t="n">
         <f aca="false">LABOR_HRS_CAR*BLENDED_RATE</f>
-        <v>0</v>
+        <v>19388.0036925463</v>
       </c>
       <c r="D12" s="11" t="n">
         <f aca="false">LABOR_HRS_MES*BLENDED_RATE</f>
-        <v>0</v>
+        <v>38660.1035720232</v>
       </c>
     </row>
   </sheetData>
@@ -1723,7 +1943,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K92"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="2" style="0" width="15"/>
@@ -1732,67 +1952,67 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="166.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="16" t="s">
-        <v>79</v>
+      <c r="A2" s="19" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17" t="s">
-        <v>81</v>
-      </c>
-      <c r="B5" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="C5" s="17" t="s">
-        <v>83</v>
-      </c>
-      <c r="D5" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="E5" s="17" t="s">
-        <v>85</v>
-      </c>
-      <c r="F5" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="G5" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="H5" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="I5" s="17" t="s">
+      <c r="A5" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="J5" s="17" t="s">
+      <c r="B5" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="K5" s="17" t="s">
+      <c r="C5" s="20" t="s">
         <v>90</v>
       </c>
+      <c r="D5" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="E5" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="F5" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="G5" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="H5" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="I5" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="J5" s="20" t="s">
+        <v>96</v>
+      </c>
+      <c r="K5" s="20" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="B6" s="14" t="n">
+      <c r="A6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6" s="17" t="n">
         <f aca="false">A6*TOM_HRS*WEEKS*(1+TOM_DIM)^A6</f>
         <v>0</v>
       </c>
-      <c r="C6" s="14" t="n">
+      <c r="C6" s="17" t="n">
         <f aca="false">MIN(B6,OWN_HRS)</f>
         <v>0</v>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="D6" s="17" t="n">
         <f aca="false">MAX(B6-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -1813,7 +2033,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="J6" s="11" t="n">
         <f aca="false">TOM_PRICE</f>
@@ -1822,18 +2042,18 @@
       <c r="K6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="n">
+      <c r="A7" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="14" t="n">
+      <c r="B7" s="17" t="n">
         <f aca="false">A7*TOM_HRS*WEEKS*(1+TOM_DIM)^A7</f>
         <v>99</v>
       </c>
-      <c r="C7" s="14" t="n">
+      <c r="C7" s="17" t="n">
         <f aca="false">MIN(B7,OWN_HRS)</f>
         <v>99</v>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="17" t="n">
         <f aca="false">MAX(B7-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -1861,24 +2081,24 @@
         <f aca="false">TOM_PRICE</f>
         <v>8800</v>
       </c>
-      <c r="K7" s="18" t="n">
+      <c r="K7" s="21" t="n">
         <f aca="false">IF(I7&gt;=TOM_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="n">
+      <c r="A8" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B8" s="17" t="n">
         <f aca="false">A8*TOM_HRS*WEEKS*(1+TOM_DIM)^A8</f>
         <v>217.8</v>
       </c>
-      <c r="C8" s="14" t="n">
+      <c r="C8" s="17" t="n">
         <f aca="false">MIN(B8,OWN_HRS)</f>
         <v>217.8</v>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="17" t="n">
         <f aca="false">MAX(B8-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -1906,24 +2126,24 @@
         <f aca="false">TOM_PRICE</f>
         <v>8800</v>
       </c>
-      <c r="K8" s="18" t="n">
+      <c r="K8" s="21" t="n">
         <f aca="false">IF(I8&gt;=TOM_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="n">
+      <c r="A9" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="17" t="n">
         <f aca="false">A9*TOM_HRS*WEEKS*(1+TOM_DIM)^A9</f>
         <v>359.37</v>
       </c>
-      <c r="C9" s="14" t="n">
+      <c r="C9" s="17" t="n">
         <f aca="false">MIN(B9,OWN_HRS)</f>
         <v>359.37</v>
       </c>
-      <c r="D9" s="14" t="n">
+      <c r="D9" s="17" t="n">
         <f aca="false">MAX(B9-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -1951,24 +2171,24 @@
         <f aca="false">TOM_PRICE</f>
         <v>8800</v>
       </c>
-      <c r="K9" s="18" t="n">
+      <c r="K9" s="21" t="n">
         <f aca="false">IF(I9&gt;=TOM_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="n">
+      <c r="A10" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="14" t="n">
+      <c r="B10" s="17" t="n">
         <f aca="false">A10*TOM_HRS*WEEKS*(1+TOM_DIM)^A10</f>
         <v>527.076</v>
       </c>
-      <c r="C10" s="14" t="n">
+      <c r="C10" s="17" t="n">
         <f aca="false">MIN(B10,OWN_HRS)</f>
         <v>527.076</v>
       </c>
-      <c r="D10" s="14" t="n">
+      <c r="D10" s="17" t="n">
         <f aca="false">MAX(B10-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -1996,24 +2216,24 @@
         <f aca="false">TOM_PRICE</f>
         <v>8800</v>
       </c>
-      <c r="K10" s="18" t="n">
+      <c r="K10" s="21" t="n">
         <f aca="false">IF(I10&gt;=TOM_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="n">
+      <c r="A11" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="B11" s="14" t="n">
+      <c r="B11" s="17" t="n">
         <f aca="false">A11*TOM_HRS*WEEKS*(1+TOM_DIM)^A11</f>
         <v>724.7295</v>
       </c>
-      <c r="C11" s="14" t="n">
+      <c r="C11" s="17" t="n">
         <f aca="false">MIN(B11,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D11" s="14" t="n">
+      <c r="D11" s="17" t="n">
         <f aca="false">MAX(B11-OWN_HRS,0)</f>
         <v>4.72950000000026</v>
       </c>
@@ -2041,24 +2261,24 @@
         <f aca="false">TOM_PRICE</f>
         <v>8800</v>
       </c>
-      <c r="K11" s="18" t="n">
+      <c r="K11" s="21" t="n">
         <f aca="false">IF(I11&gt;=TOM_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="n">
+      <c r="A12" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="B12" s="14" t="n">
+      <c r="B12" s="17" t="n">
         <f aca="false">A12*TOM_HRS*WEEKS*(1+TOM_DIM)^A12</f>
         <v>956.64294</v>
       </c>
-      <c r="C12" s="14" t="n">
+      <c r="C12" s="17" t="n">
         <f aca="false">MIN(B12,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D12" s="14" t="n">
+      <c r="D12" s="17" t="n">
         <f aca="false">MAX(B12-OWN_HRS,0)</f>
         <v>236.64294</v>
       </c>
@@ -2086,24 +2306,24 @@
         <f aca="false">TOM_PRICE</f>
         <v>8800</v>
       </c>
-      <c r="K12" s="18" t="n">
+      <c r="K12" s="21" t="n">
         <f aca="false">IF(I12&gt;=TOM_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="18" t="n">
+      <c r="A13" s="21" t="n">
         <v>7</v>
       </c>
-      <c r="B13" s="14" t="n">
+      <c r="B13" s="17" t="n">
         <f aca="false">A13*TOM_HRS*WEEKS*(1+TOM_DIM)^A13</f>
         <v>1227.691773</v>
       </c>
-      <c r="C13" s="14" t="n">
+      <c r="C13" s="17" t="n">
         <f aca="false">MIN(B13,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D13" s="14" t="n">
+      <c r="D13" s="17" t="n">
         <f aca="false">MAX(B13-OWN_HRS,0)</f>
         <v>507.691773000001</v>
       </c>
@@ -2131,24 +2351,24 @@
         <f aca="false">TOM_PRICE</f>
         <v>8800</v>
       </c>
-      <c r="K13" s="18" t="n">
+      <c r="K13" s="21" t="n">
         <f aca="false">IF(I13&gt;=TOM_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="18" t="n">
+      <c r="A14" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="B14" s="14" t="n">
+      <c r="B14" s="17" t="n">
         <f aca="false">A14*TOM_HRS*WEEKS*(1+TOM_DIM)^A14</f>
         <v>1543.3839432</v>
       </c>
-      <c r="C14" s="14" t="n">
+      <c r="C14" s="17" t="n">
         <f aca="false">MIN(B14,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D14" s="14" t="n">
+      <c r="D14" s="17" t="n">
         <f aca="false">MAX(B14-OWN_HRS,0)</f>
         <v>823.383943200001</v>
       </c>
@@ -2176,24 +2396,24 @@
         <f aca="false">TOM_PRICE</f>
         <v>8800</v>
       </c>
-      <c r="K14" s="18" t="n">
+      <c r="K14" s="21" t="n">
         <f aca="false">IF(I14&gt;=TOM_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="18" t="n">
+      <c r="A15" s="21" t="n">
         <v>9</v>
       </c>
-      <c r="B15" s="14" t="n">
+      <c r="B15" s="17" t="n">
         <f aca="false">A15*TOM_HRS*WEEKS*(1+TOM_DIM)^A15</f>
         <v>1909.93762971</v>
       </c>
-      <c r="C15" s="14" t="n">
+      <c r="C15" s="17" t="n">
         <f aca="false">MIN(B15,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D15" s="14" t="n">
+      <c r="D15" s="17" t="n">
         <f aca="false">MAX(B15-OWN_HRS,0)</f>
         <v>1189.93762971</v>
       </c>
@@ -2221,24 +2441,24 @@
         <f aca="false">TOM_PRICE</f>
         <v>8800</v>
       </c>
-      <c r="K15" s="18" t="n">
+      <c r="K15" s="21" t="n">
         <f aca="false">IF(I15&gt;=TOM_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="18" t="n">
+      <c r="A16" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="B16" s="14" t="n">
+      <c r="B16" s="17" t="n">
         <f aca="false">A16*TOM_HRS*WEEKS*(1+TOM_DIM)^A16</f>
         <v>2334.36821409</v>
       </c>
-      <c r="C16" s="14" t="n">
+      <c r="C16" s="17" t="n">
         <f aca="false">MIN(B16,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D16" s="14" t="n">
+      <c r="D16" s="17" t="n">
         <f aca="false">MAX(B16-OWN_HRS,0)</f>
         <v>1614.36821409</v>
       </c>
@@ -2266,24 +2486,24 @@
         <f aca="false">TOM_PRICE</f>
         <v>8800</v>
       </c>
-      <c r="K16" s="18" t="n">
+      <c r="K16" s="21" t="n">
         <f aca="false">IF(I16&gt;=TOM_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="18" t="n">
+      <c r="A17" s="21" t="n">
         <v>11</v>
       </c>
-      <c r="B17" s="14" t="n">
+      <c r="B17" s="17" t="n">
         <f aca="false">A17*TOM_HRS*WEEKS*(1+TOM_DIM)^A17</f>
         <v>2824.5855390489</v>
       </c>
-      <c r="C17" s="14" t="n">
+      <c r="C17" s="17" t="n">
         <f aca="false">MIN(B17,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D17" s="14" t="n">
+      <c r="D17" s="17" t="n">
         <f aca="false">MAX(B17-OWN_HRS,0)</f>
         <v>2104.5855390489</v>
       </c>
@@ -2311,24 +2531,24 @@
         <f aca="false">TOM_PRICE</f>
         <v>8800</v>
       </c>
-      <c r="K17" s="18" t="n">
+      <c r="K17" s="21" t="n">
         <f aca="false">IF(I17&gt;=TOM_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="18" t="n">
+      <c r="A18" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="B18" s="14" t="n">
+      <c r="B18" s="17" t="n">
         <f aca="false">A18*TOM_HRS*WEEKS*(1+TOM_DIM)^A18</f>
         <v>3389.50264685868</v>
       </c>
-      <c r="C18" s="14" t="n">
+      <c r="C18" s="17" t="n">
         <f aca="false">MIN(B18,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D18" s="14" t="n">
+      <c r="D18" s="17" t="n">
         <f aca="false">MAX(B18-OWN_HRS,0)</f>
         <v>2669.50264685868</v>
       </c>
@@ -2356,24 +2576,24 @@
         <f aca="false">TOM_PRICE</f>
         <v>8800</v>
       </c>
-      <c r="K18" s="18" t="n">
+      <c r="K18" s="21" t="n">
         <f aca="false">IF(I18&gt;=TOM_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="18" t="n">
+      <c r="A19" s="21" t="n">
         <v>13</v>
       </c>
-      <c r="B19" s="14" t="n">
+      <c r="B19" s="17" t="n">
         <f aca="false">A19*TOM_HRS*WEEKS*(1+TOM_DIM)^A19</f>
         <v>4039.15732083993</v>
       </c>
-      <c r="C19" s="14" t="n">
+      <c r="C19" s="17" t="n">
         <f aca="false">MIN(B19,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D19" s="14" t="n">
+      <c r="D19" s="17" t="n">
         <f aca="false">MAX(B19-OWN_HRS,0)</f>
         <v>3319.15732083993</v>
       </c>
@@ -2401,24 +2621,24 @@
         <f aca="false">TOM_PRICE</f>
         <v>8800</v>
       </c>
-      <c r="K19" s="18" t="n">
+      <c r="K19" s="21" t="n">
         <f aca="false">IF(I19&gt;=TOM_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="18" t="n">
+      <c r="A20" s="21" t="n">
         <v>14</v>
       </c>
-      <c r="B20" s="14" t="n">
+      <c r="B20" s="17" t="n">
         <f aca="false">A20*TOM_HRS*WEEKS*(1+TOM_DIM)^A20</f>
         <v>4784.84790314884</v>
       </c>
-      <c r="C20" s="14" t="n">
+      <c r="C20" s="17" t="n">
         <f aca="false">MIN(B20,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D20" s="14" t="n">
+      <c r="D20" s="17" t="n">
         <f aca="false">MAX(B20-OWN_HRS,0)</f>
         <v>4064.84790314884</v>
       </c>
@@ -2446,24 +2666,24 @@
         <f aca="false">TOM_PRICE</f>
         <v>8800</v>
       </c>
-      <c r="K20" s="18" t="n">
+      <c r="K20" s="21" t="n">
         <f aca="false">IF(I20&gt;=TOM_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="18" t="n">
+      <c r="A21" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="B21" s="14" t="n">
+      <c r="B21" s="17" t="n">
         <f aca="false">A21*TOM_HRS*WEEKS*(1+TOM_DIM)^A21</f>
         <v>5639.28502871114</v>
       </c>
-      <c r="C21" s="14" t="n">
+      <c r="C21" s="17" t="n">
         <f aca="false">MIN(B21,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D21" s="14" t="n">
+      <c r="D21" s="17" t="n">
         <f aca="false">MAX(B21-OWN_HRS,0)</f>
         <v>4919.28502871114</v>
       </c>
@@ -2491,24 +2711,24 @@
         <f aca="false">TOM_PRICE</f>
         <v>8800</v>
       </c>
-      <c r="K21" s="18" t="n">
+      <c r="K21" s="21" t="n">
         <f aca="false">IF(I21&gt;=TOM_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="18" t="n">
+      <c r="A22" s="21" t="n">
         <v>16</v>
       </c>
-      <c r="B22" s="14" t="n">
+      <c r="B22" s="17" t="n">
         <f aca="false">A22*TOM_HRS*WEEKS*(1+TOM_DIM)^A22</f>
         <v>6616.7611003544</v>
       </c>
-      <c r="C22" s="14" t="n">
+      <c r="C22" s="17" t="n">
         <f aca="false">MIN(B22,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D22" s="14" t="n">
+      <c r="D22" s="17" t="n">
         <f aca="false">MAX(B22-OWN_HRS,0)</f>
         <v>5896.7611003544</v>
       </c>
@@ -2536,24 +2756,24 @@
         <f aca="false">TOM_PRICE</f>
         <v>8800</v>
       </c>
-      <c r="K22" s="18" t="n">
+      <c r="K22" s="21" t="n">
         <f aca="false">IF(I22&gt;=TOM_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="18" t="n">
+      <c r="A23" s="21" t="n">
         <v>17</v>
       </c>
-      <c r="B23" s="14" t="n">
+      <c r="B23" s="17" t="n">
         <f aca="false">A23*TOM_HRS*WEEKS*(1+TOM_DIM)^A23</f>
         <v>7733.33953603921</v>
       </c>
-      <c r="C23" s="14" t="n">
+      <c r="C23" s="17" t="n">
         <f aca="false">MIN(B23,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D23" s="14" t="n">
+      <c r="D23" s="17" t="n">
         <f aca="false">MAX(B23-OWN_HRS,0)</f>
         <v>7013.33953603921</v>
       </c>
@@ -2581,24 +2801,24 @@
         <f aca="false">TOM_PRICE</f>
         <v>8800</v>
       </c>
-      <c r="K23" s="18" t="n">
+      <c r="K23" s="21" t="n">
         <f aca="false">IF(I23&gt;=TOM_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="18" t="n">
+      <c r="A24" s="21" t="n">
         <v>18</v>
       </c>
-      <c r="B24" s="14" t="n">
+      <c r="B24" s="17" t="n">
         <f aca="false">A24*TOM_HRS*WEEKS*(1+TOM_DIM)^A24</f>
         <v>9007.06604785743</v>
       </c>
-      <c r="C24" s="14" t="n">
+      <c r="C24" s="17" t="n">
         <f aca="false">MIN(B24,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D24" s="14" t="n">
+      <c r="D24" s="17" t="n">
         <f aca="false">MAX(B24-OWN_HRS,0)</f>
         <v>8287.06604785743</v>
       </c>
@@ -2626,24 +2846,24 @@
         <f aca="false">TOM_PRICE</f>
         <v>8800</v>
       </c>
-      <c r="K24" s="18" t="n">
+      <c r="K24" s="21" t="n">
         <f aca="false">IF(I24&gt;=TOM_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="18" t="n">
+      <c r="A25" s="21" t="n">
         <v>19</v>
       </c>
-      <c r="B25" s="14" t="n">
+      <c r="B25" s="17" t="n">
         <f aca="false">A25*TOM_HRS*WEEKS*(1+TOM_DIM)^A25</f>
         <v>10458.2044666789</v>
       </c>
-      <c r="C25" s="14" t="n">
+      <c r="C25" s="17" t="n">
         <f aca="false">MIN(B25,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D25" s="14" t="n">
+      <c r="D25" s="17" t="n">
         <f aca="false">MAX(B25-OWN_HRS,0)</f>
         <v>9738.2044666789</v>
       </c>
@@ -2671,24 +2891,24 @@
         <f aca="false">TOM_PRICE</f>
         <v>8800</v>
       </c>
-      <c r="K25" s="18" t="n">
+      <c r="K25" s="21" t="n">
         <f aca="false">IF(I25&gt;=TOM_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="18" t="n">
+      <c r="A26" s="21" t="n">
         <v>20</v>
       </c>
-      <c r="B26" s="14" t="n">
+      <c r="B26" s="17" t="n">
         <f aca="false">A26*TOM_HRS*WEEKS*(1+TOM_DIM)^A26</f>
         <v>12109.4999087861</v>
       </c>
-      <c r="C26" s="14" t="n">
+      <c r="C26" s="17" t="n">
         <f aca="false">MIN(B26,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D26" s="14" t="n">
+      <c r="D26" s="17" t="n">
         <f aca="false">MAX(B26-OWN_HRS,0)</f>
         <v>11389.4999087861</v>
       </c>
@@ -2716,73 +2936,73 @@
         <f aca="false">TOM_PRICE</f>
         <v>8800</v>
       </c>
-      <c r="K26" s="18" t="n">
+      <c r="K26" s="21" t="n">
         <f aca="false">IF(I26&gt;=TOM_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="B28" s="19" t="n">
+        <v>99</v>
+      </c>
+      <c r="B28" s="22" t="n">
         <f aca="false">IF(ISNA(MATCH(1,'Marginal Cost Schedules'!$K$7:$K$26,0)),TOM_CAP,MATCH(1,'Marginal Cost Schedules'!$K$7:$K$26,0)-1)</f>
         <v>10</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="B32" s="20" t="s">
+        <v>89</v>
+      </c>
+      <c r="C32" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="D32" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="E32" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="F32" s="20" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="17" t="s">
-        <v>81</v>
-      </c>
-      <c r="B32" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="C32" s="17" t="s">
-        <v>83</v>
-      </c>
-      <c r="D32" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="E32" s="17" t="s">
-        <v>85</v>
-      </c>
-      <c r="F32" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="G32" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="H32" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="I32" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="J32" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="K32" s="17" t="s">
-        <v>90</v>
+      <c r="G32" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="H32" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="I32" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="J32" s="20" t="s">
+        <v>96</v>
+      </c>
+      <c r="K32" s="20" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="B33" s="14" t="n">
+      <c r="A33" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="B33" s="17" t="n">
         <f aca="false">A33*CAR_HRS*WEEKS*(1+CAR_DIM)^A33</f>
         <v>0</v>
       </c>
-      <c r="C33" s="14" t="n">
+      <c r="C33" s="17" t="n">
         <f aca="false">MIN(B33,OWN_HRS)</f>
         <v>0</v>
       </c>
-      <c r="D33" s="14" t="n">
+      <c r="D33" s="17" t="n">
         <f aca="false">MAX(B33-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -2803,7 +3023,7 @@
         <v>0</v>
       </c>
       <c r="I33" s="5" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="J33" s="11" t="n">
         <f aca="false">CAR_PRICE</f>
@@ -2812,18 +3032,18 @@
       <c r="K33" s="5"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="18" t="n">
+      <c r="A34" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="B34" s="14" t="n">
+      <c r="B34" s="17" t="n">
         <f aca="false">A34*CAR_HRS*WEEKS*(1+CAR_DIM)^A34</f>
         <v>30.7377</v>
       </c>
-      <c r="C34" s="14" t="n">
+      <c r="C34" s="17" t="n">
         <f aca="false">MIN(B34,OWN_HRS)</f>
         <v>30.7377</v>
       </c>
-      <c r="D34" s="14" t="n">
+      <c r="D34" s="17" t="n">
         <f aca="false">MAX(B34-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -2851,24 +3071,24 @@
         <f aca="false">CAR_PRICE</f>
         <v>2094</v>
       </c>
-      <c r="K34" s="18" t="n">
+      <c r="K34" s="21" t="n">
         <f aca="false">IF(I34&gt;=CAR_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="18" t="n">
+      <c r="A35" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="B35" s="14" t="n">
+      <c r="B35" s="17" t="n">
         <f aca="false">A35*CAR_HRS*WEEKS*(1+CAR_DIM)^A35</f>
         <v>63.012285</v>
       </c>
-      <c r="C35" s="14" t="n">
+      <c r="C35" s="17" t="n">
         <f aca="false">MIN(B35,OWN_HRS)</f>
         <v>63.012285</v>
       </c>
-      <c r="D35" s="14" t="n">
+      <c r="D35" s="17" t="n">
         <f aca="false">MAX(B35-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -2896,24 +3116,24 @@
         <f aca="false">CAR_PRICE</f>
         <v>2094</v>
       </c>
-      <c r="K35" s="18" t="n">
+      <c r="K35" s="21" t="n">
         <f aca="false">IF(I35&gt;=CAR_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="18" t="n">
+      <c r="A36" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="B36" s="14" t="n">
+      <c r="B36" s="17" t="n">
         <f aca="false">A36*CAR_HRS*WEEKS*(1+CAR_DIM)^A36</f>
         <v>96.8813881875</v>
       </c>
-      <c r="C36" s="14" t="n">
+      <c r="C36" s="17" t="n">
         <f aca="false">MIN(B36,OWN_HRS)</f>
         <v>96.8813881875</v>
       </c>
-      <c r="D36" s="14" t="n">
+      <c r="D36" s="17" t="n">
         <f aca="false">MAX(B36-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -2941,24 +3161,24 @@
         <f aca="false">CAR_PRICE</f>
         <v>2094</v>
       </c>
-      <c r="K36" s="18" t="n">
+      <c r="K36" s="21" t="n">
         <f aca="false">IF(I36&gt;=CAR_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="18" t="n">
+      <c r="A37" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="B37" s="14" t="n">
+      <c r="B37" s="17" t="n">
         <f aca="false">A37*CAR_HRS*WEEKS*(1+CAR_DIM)^A37</f>
         <v>132.40456385625</v>
       </c>
-      <c r="C37" s="14" t="n">
+      <c r="C37" s="17" t="n">
         <f aca="false">MIN(B37,OWN_HRS)</f>
         <v>132.40456385625</v>
       </c>
-      <c r="D37" s="14" t="n">
+      <c r="D37" s="17" t="n">
         <f aca="false">MAX(B37-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -2986,24 +3206,24 @@
         <f aca="false">CAR_PRICE</f>
         <v>2094</v>
       </c>
-      <c r="K37" s="18" t="n">
+      <c r="K37" s="21" t="n">
         <f aca="false">IF(I37&gt;=CAR_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="18" t="n">
+      <c r="A38" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="B38" s="14" t="n">
+      <c r="B38" s="17" t="n">
         <f aca="false">A38*CAR_HRS*WEEKS*(1+CAR_DIM)^A38</f>
         <v>169.64334744082</v>
       </c>
-      <c r="C38" s="14" t="n">
+      <c r="C38" s="17" t="n">
         <f aca="false">MIN(B38,OWN_HRS)</f>
         <v>169.64334744082</v>
       </c>
-      <c r="D38" s="14" t="n">
+      <c r="D38" s="17" t="n">
         <f aca="false">MAX(B38-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -3031,24 +3251,24 @@
         <f aca="false">CAR_PRICE</f>
         <v>2094</v>
       </c>
-      <c r="K38" s="18" t="n">
+      <c r="K38" s="21" t="n">
         <f aca="false">IF(I38&gt;=CAR_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="18" t="n">
+      <c r="A39" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="B39" s="14" t="n">
+      <c r="B39" s="17" t="n">
         <f aca="false">A39*CAR_HRS*WEEKS*(1+CAR_DIM)^A39</f>
         <v>208.661317352209</v>
       </c>
-      <c r="C39" s="14" t="n">
+      <c r="C39" s="17" t="n">
         <f aca="false">MIN(B39,OWN_HRS)</f>
         <v>208.661317352209</v>
       </c>
-      <c r="D39" s="14" t="n">
+      <c r="D39" s="17" t="n">
         <f aca="false">MAX(B39-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -3076,24 +3296,24 @@
         <f aca="false">CAR_PRICE</f>
         <v>2094</v>
       </c>
-      <c r="K39" s="18" t="n">
+      <c r="K39" s="21" t="n">
         <f aca="false">IF(I39&gt;=CAR_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="18" t="n">
+      <c r="A40" s="21" t="n">
         <v>7</v>
       </c>
-      <c r="B40" s="14" t="n">
+      <c r="B40" s="17" t="n">
         <f aca="false">A40*CAR_HRS*WEEKS*(1+CAR_DIM)^A40</f>
         <v>249.524158667016</v>
       </c>
-      <c r="C40" s="14" t="n">
+      <c r="C40" s="17" t="n">
         <f aca="false">MIN(B40,OWN_HRS)</f>
         <v>249.524158667016</v>
       </c>
-      <c r="D40" s="14" t="n">
+      <c r="D40" s="17" t="n">
         <f aca="false">MAX(B40-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -3121,24 +3341,24 @@
         <f aca="false">CAR_PRICE</f>
         <v>2094</v>
       </c>
-      <c r="K40" s="18" t="n">
+      <c r="K40" s="21" t="n">
         <f aca="false">IF(I40&gt;=CAR_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="18" t="n">
+      <c r="A41" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="B41" s="14" t="n">
+      <c r="B41" s="17" t="n">
         <f aca="false">A41*CAR_HRS*WEEKS*(1+CAR_DIM)^A41</f>
         <v>292.299728724219</v>
       </c>
-      <c r="C41" s="14" t="n">
+      <c r="C41" s="17" t="n">
         <f aca="false">MIN(B41,OWN_HRS)</f>
         <v>292.299728724219</v>
       </c>
-      <c r="D41" s="14" t="n">
+      <c r="D41" s="17" t="n">
         <f aca="false">MAX(B41-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -3166,24 +3386,24 @@
         <f aca="false">CAR_PRICE</f>
         <v>2094</v>
       </c>
-      <c r="K41" s="18" t="n">
+      <c r="K41" s="21" t="n">
         <f aca="false">IF(I41&gt;=CAR_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="18" t="n">
+      <c r="A42" s="21" t="n">
         <v>9</v>
       </c>
-      <c r="B42" s="14" t="n">
+      <c r="B42" s="17" t="n">
         <f aca="false">A42*CAR_HRS*WEEKS*(1+CAR_DIM)^A42</f>
         <v>337.058124685115</v>
       </c>
-      <c r="C42" s="14" t="n">
+      <c r="C42" s="17" t="n">
         <f aca="false">MIN(B42,OWN_HRS)</f>
         <v>337.058124685115</v>
       </c>
-      <c r="D42" s="14" t="n">
+      <c r="D42" s="17" t="n">
         <f aca="false">MAX(B42-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -3211,24 +3431,24 @@
         <f aca="false">CAR_PRICE</f>
         <v>2094</v>
       </c>
-      <c r="K42" s="18" t="n">
+      <c r="K42" s="21" t="n">
         <f aca="false">IF(I42&gt;=CAR_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="18" t="n">
+      <c r="A43" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="B43" s="14" t="n">
+      <c r="B43" s="17" t="n">
         <f aca="false">A43*CAR_HRS*WEEKS*(1+CAR_DIM)^A43</f>
         <v>383.871753113603</v>
       </c>
-      <c r="C43" s="14" t="n">
+      <c r="C43" s="17" t="n">
         <f aca="false">MIN(B43,OWN_HRS)</f>
         <v>383.871753113603</v>
       </c>
-      <c r="D43" s="14" t="n">
+      <c r="D43" s="17" t="n">
         <f aca="false">MAX(B43-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -3256,24 +3476,24 @@
         <f aca="false">CAR_PRICE</f>
         <v>2094</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="K43" s="21" t="n">
         <f aca="false">IF(I43&gt;=CAR_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="18" t="n">
+      <c r="A44" s="21" t="n">
         <v>11</v>
       </c>
-      <c r="B44" s="14" t="n">
+      <c r="B44" s="17" t="n">
         <f aca="false">A44*CAR_HRS*WEEKS*(1+CAR_DIM)^A44</f>
         <v>432.815401635588</v>
       </c>
-      <c r="C44" s="14" t="n">
+      <c r="C44" s="17" t="n">
         <f aca="false">MIN(B44,OWN_HRS)</f>
         <v>432.815401635588</v>
       </c>
-      <c r="D44" s="14" t="n">
+      <c r="D44" s="17" t="n">
         <f aca="false">MAX(B44-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -3301,24 +3521,24 @@
         <f aca="false">CAR_PRICE</f>
         <v>2094</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="K44" s="21" t="n">
         <f aca="false">IF(I44&gt;=CAR_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="18" t="n">
+      <c r="A45" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="B45" s="14" t="n">
+      <c r="B45" s="17" t="n">
         <f aca="false">A45*CAR_HRS*WEEKS*(1+CAR_DIM)^A45</f>
         <v>483.966312737975</v>
       </c>
-      <c r="C45" s="14" t="n">
+      <c r="C45" s="17" t="n">
         <f aca="false">MIN(B45,OWN_HRS)</f>
         <v>483.966312737975</v>
       </c>
-      <c r="D45" s="14" t="n">
+      <c r="D45" s="17" t="n">
         <f aca="false">MAX(B45-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -3346,24 +3566,24 @@
         <f aca="false">CAR_PRICE</f>
         <v>2094</v>
       </c>
-      <c r="K45" s="18" t="n">
+      <c r="K45" s="21" t="n">
         <f aca="false">IF(I45&gt;=CAR_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="18" t="n">
+      <c r="A46" s="21" t="n">
         <v>13</v>
       </c>
-      <c r="B46" s="14" t="n">
+      <c r="B46" s="17" t="n">
         <f aca="false">A46*CAR_HRS*WEEKS*(1+CAR_DIM)^A46</f>
         <v>537.40425976946</v>
       </c>
-      <c r="C46" s="14" t="n">
+      <c r="C46" s="17" t="n">
         <f aca="false">MIN(B46,OWN_HRS)</f>
         <v>537.40425976946</v>
       </c>
-      <c r="D46" s="14" t="n">
+      <c r="D46" s="17" t="n">
         <f aca="false">MAX(B46-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -3391,24 +3611,24 @@
         <f aca="false">CAR_PRICE</f>
         <v>2094</v>
       </c>
-      <c r="K46" s="18" t="n">
+      <c r="K46" s="21" t="n">
         <f aca="false">IF(I46&gt;=CAR_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="18" t="n">
+      <c r="A47" s="21" t="n">
         <v>14</v>
       </c>
-      <c r="B47" s="14" t="n">
+      <c r="B47" s="17" t="n">
         <f aca="false">A47*CAR_HRS*WEEKS*(1+CAR_DIM)^A47</f>
         <v>593.211625207058</v>
       </c>
-      <c r="C47" s="14" t="n">
+      <c r="C47" s="17" t="n">
         <f aca="false">MIN(B47,OWN_HRS)</f>
         <v>593.211625207058</v>
       </c>
-      <c r="D47" s="14" t="n">
+      <c r="D47" s="17" t="n">
         <f aca="false">MAX(B47-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -3436,24 +3656,24 @@
         <f aca="false">CAR_PRICE</f>
         <v>2094</v>
       </c>
-      <c r="K47" s="18" t="n">
+      <c r="K47" s="21" t="n">
         <f aca="false">IF(I47&gt;=CAR_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="18" t="n">
+      <c r="A48" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="B48" s="14" t="n">
+      <c r="B48" s="17" t="n">
         <f aca="false">A48*CAR_HRS*WEEKS*(1+CAR_DIM)^A48</f>
         <v>651.47348125418</v>
       </c>
-      <c r="C48" s="14" t="n">
+      <c r="C48" s="17" t="n">
         <f aca="false">MIN(B48,OWN_HRS)</f>
         <v>651.47348125418</v>
       </c>
-      <c r="D48" s="14" t="n">
+      <c r="D48" s="17" t="n">
         <f aca="false">MAX(B48-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -3481,24 +3701,24 @@
         <f aca="false">CAR_PRICE</f>
         <v>2094</v>
       </c>
-      <c r="K48" s="18" t="n">
+      <c r="K48" s="21" t="n">
         <f aca="false">IF(I48&gt;=CAR_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="18" t="n">
+      <c r="A49" s="21" t="n">
         <v>16</v>
       </c>
-      <c r="B49" s="14" t="n">
+      <c r="B49" s="17" t="n">
         <f aca="false">A49*CAR_HRS*WEEKS*(1+CAR_DIM)^A49</f>
         <v>712.277672837903</v>
       </c>
-      <c r="C49" s="14" t="n">
+      <c r="C49" s="17" t="n">
         <f aca="false">MIN(B49,OWN_HRS)</f>
         <v>712.277672837903</v>
       </c>
-      <c r="D49" s="14" t="n">
+      <c r="D49" s="17" t="n">
         <f aca="false">MAX(B49-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -3526,24 +3746,24 @@
         <f aca="false">CAR_PRICE</f>
         <v>2094</v>
       </c>
-      <c r="K49" s="18" t="n">
+      <c r="K49" s="21" t="n">
         <f aca="false">IF(I49&gt;=CAR_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="18" t="n">
+      <c r="A50" s="21" t="n">
         <v>17</v>
       </c>
-      <c r="B50" s="14" t="n">
+      <c r="B50" s="17" t="n">
         <f aca="false">A50*CAR_HRS*WEEKS*(1+CAR_DIM)^A50</f>
         <v>775.714903075029</v>
       </c>
-      <c r="C50" s="14" t="n">
+      <c r="C50" s="17" t="n">
         <f aca="false">MIN(B50,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D50" s="14" t="n">
+      <c r="D50" s="17" t="n">
         <f aca="false">MAX(B50-OWN_HRS,0)</f>
         <v>55.7149030750287</v>
       </c>
@@ -3571,24 +3791,24 @@
         <f aca="false">CAR_PRICE</f>
         <v>2094</v>
       </c>
-      <c r="K50" s="18" t="n">
+      <c r="K50" s="21" t="n">
         <f aca="false">IF(I50&gt;=CAR_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="18" t="n">
+      <c r="A51" s="21" t="n">
         <v>18</v>
       </c>
-      <c r="B51" s="14" t="n">
+      <c r="B51" s="17" t="n">
         <f aca="false">A51*CAR_HRS*WEEKS*(1+CAR_DIM)^A51</f>
         <v>841.878821278487</v>
       </c>
-      <c r="C51" s="14" t="n">
+      <c r="C51" s="17" t="n">
         <f aca="false">MIN(B51,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D51" s="14" t="n">
+      <c r="D51" s="17" t="n">
         <f aca="false">MAX(B51-OWN_HRS,0)</f>
         <v>121.878821278487</v>
       </c>
@@ -3616,24 +3836,24 @@
         <f aca="false">CAR_PRICE</f>
         <v>2094</v>
       </c>
-      <c r="K51" s="18" t="n">
+      <c r="K51" s="21" t="n">
         <f aca="false">IF(I51&gt;=CAR_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="18" t="n">
+      <c r="A52" s="21" t="n">
         <v>19</v>
       </c>
-      <c r="B52" s="14" t="n">
+      <c r="B52" s="17" t="n">
         <f aca="false">A52*CAR_HRS*WEEKS*(1+CAR_DIM)^A52</f>
         <v>910.866113577696</v>
       </c>
-      <c r="C52" s="14" t="n">
+      <c r="C52" s="17" t="n">
         <f aca="false">MIN(B52,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D52" s="14" t="n">
+      <c r="D52" s="17" t="n">
         <f aca="false">MAX(B52-OWN_HRS,0)</f>
         <v>190.866113577696</v>
       </c>
@@ -3661,24 +3881,24 @@
         <f aca="false">CAR_PRICE</f>
         <v>2094</v>
       </c>
-      <c r="K52" s="18" t="n">
+      <c r="K52" s="21" t="n">
         <f aca="false">IF(I52&gt;=CAR_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="18" t="n">
+      <c r="A53" s="21" t="n">
         <v>20</v>
       </c>
-      <c r="B53" s="14" t="n">
+      <c r="B53" s="17" t="n">
         <f aca="false">A53*CAR_HRS*WEEKS*(1+CAR_DIM)^A53</f>
         <v>982.776596228567</v>
       </c>
-      <c r="C53" s="14" t="n">
+      <c r="C53" s="17" t="n">
         <f aca="false">MIN(B53,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D53" s="14" t="n">
+      <c r="D53" s="17" t="n">
         <f aca="false">MAX(B53-OWN_HRS,0)</f>
         <v>262.776596228567</v>
       </c>
@@ -3706,73 +3926,73 @@
         <f aca="false">CAR_PRICE</f>
         <v>2094</v>
       </c>
-      <c r="K53" s="18" t="n">
+      <c r="K53" s="21" t="n">
         <f aca="false">IF(I53&gt;=CAR_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B55" s="19" t="n">
+        <v>101</v>
+      </c>
+      <c r="B55" s="22" t="n">
         <f aca="false">IF(ISNA(MATCH(1,'Marginal Cost Schedules'!$K$34:$K$53,0)),CAR_CAP,MATCH(1,'Marginal Cost Schedules'!$K$34:$K$53,0)-1)</f>
         <v>10</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="9" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="17" t="s">
-        <v>81</v>
-      </c>
-      <c r="B59" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="C59" s="17" t="s">
-        <v>83</v>
-      </c>
-      <c r="D59" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="E59" s="17" t="s">
-        <v>85</v>
-      </c>
-      <c r="F59" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="G59" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="H59" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="I59" s="17" t="s">
+      <c r="A59" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="J59" s="17" t="s">
+      <c r="B59" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="K59" s="17" t="s">
+      <c r="C59" s="20" t="s">
         <v>90</v>
       </c>
+      <c r="D59" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="E59" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="F59" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="G59" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="H59" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="I59" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="J59" s="20" t="s">
+        <v>96</v>
+      </c>
+      <c r="K59" s="20" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="B60" s="14" t="n">
+      <c r="A60" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="B60" s="17" t="n">
         <f aca="false">A60*MES_HRS*WEEKS*(1+MES_DIM)^A60</f>
         <v>0</v>
       </c>
-      <c r="C60" s="14" t="n">
+      <c r="C60" s="17" t="n">
         <f aca="false">MIN(B60,OWN_HRS)</f>
         <v>0</v>
       </c>
-      <c r="D60" s="14" t="n">
+      <c r="D60" s="17" t="n">
         <f aca="false">MAX(B60-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -3793,7 +4013,7 @@
         <v>0</v>
       </c>
       <c r="I60" s="5" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="J60" s="11" t="n">
         <f aca="false">MES_PRICE</f>
@@ -3802,18 +4022,18 @@
       <c r="K60" s="5"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="18" t="n">
+      <c r="A61" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="B61" s="14" t="n">
+      <c r="B61" s="17" t="n">
         <f aca="false">A61*MES_HRS*WEEKS*(1+MES_DIM)^A61</f>
         <v>45.5625</v>
       </c>
-      <c r="C61" s="14" t="n">
+      <c r="C61" s="17" t="n">
         <f aca="false">MIN(B61,OWN_HRS)</f>
         <v>45.5625</v>
       </c>
-      <c r="D61" s="14" t="n">
+      <c r="D61" s="17" t="n">
         <f aca="false">MAX(B61-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -3841,24 +4061,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K61" s="18" t="n">
+      <c r="K61" s="21" t="n">
         <f aca="false">IF(I61&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="18" t="n">
+      <c r="A62" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="B62" s="14" t="n">
+      <c r="B62" s="17" t="n">
         <f aca="false">A62*MES_HRS*WEEKS*(1+MES_DIM)^A62</f>
         <v>92.2640625</v>
       </c>
-      <c r="C62" s="14" t="n">
+      <c r="C62" s="17" t="n">
         <f aca="false">MIN(B62,OWN_HRS)</f>
         <v>92.2640625</v>
       </c>
-      <c r="D62" s="14" t="n">
+      <c r="D62" s="17" t="n">
         <f aca="false">MAX(B62-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -3886,24 +4106,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K62" s="18" t="n">
+      <c r="K62" s="21" t="n">
         <f aca="false">IF(I62&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="18" t="n">
+      <c r="A63" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="B63" s="14" t="n">
+      <c r="B63" s="17" t="n">
         <f aca="false">A63*MES_HRS*WEEKS*(1+MES_DIM)^A63</f>
         <v>140.126044921875</v>
       </c>
-      <c r="C63" s="14" t="n">
+      <c r="C63" s="17" t="n">
         <f aca="false">MIN(B63,OWN_HRS)</f>
         <v>140.126044921875</v>
       </c>
-      <c r="D63" s="14" t="n">
+      <c r="D63" s="17" t="n">
         <f aca="false">MAX(B63-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -3931,24 +4151,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K63" s="18" t="n">
+      <c r="K63" s="21" t="n">
         <f aca="false">IF(I63&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="18" t="n">
+      <c r="A64" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="B64" s="14" t="n">
+      <c r="B64" s="17" t="n">
         <f aca="false">A64*MES_HRS*WEEKS*(1+MES_DIM)^A64</f>
         <v>189.170160644531</v>
       </c>
-      <c r="C64" s="14" t="n">
+      <c r="C64" s="17" t="n">
         <f aca="false">MIN(B64,OWN_HRS)</f>
         <v>189.170160644531</v>
       </c>
-      <c r="D64" s="14" t="n">
+      <c r="D64" s="17" t="n">
         <f aca="false">MAX(B64-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -3976,24 +4196,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K64" s="18" t="n">
+      <c r="K64" s="21" t="n">
         <f aca="false">IF(I64&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="18" t="n">
+      <c r="A65" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="B65" s="14" t="n">
+      <c r="B65" s="17" t="n">
         <f aca="false">A65*MES_HRS*WEEKS*(1+MES_DIM)^A65</f>
         <v>239.418484565735</v>
       </c>
-      <c r="C65" s="14" t="n">
+      <c r="C65" s="17" t="n">
         <f aca="false">MIN(B65,OWN_HRS)</f>
         <v>239.418484565735</v>
       </c>
-      <c r="D65" s="14" t="n">
+      <c r="D65" s="17" t="n">
         <f aca="false">MAX(B65-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -4021,24 +4241,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K65" s="18" t="n">
+      <c r="K65" s="21" t="n">
         <f aca="false">IF(I65&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="18" t="n">
+      <c r="A66" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="B66" s="14" t="n">
+      <c r="B66" s="17" t="n">
         <f aca="false">A66*MES_HRS*WEEKS*(1+MES_DIM)^A66</f>
         <v>290.893458747368</v>
       </c>
-      <c r="C66" s="14" t="n">
+      <c r="C66" s="17" t="n">
         <f aca="false">MIN(B66,OWN_HRS)</f>
         <v>290.893458747368</v>
       </c>
-      <c r="D66" s="14" t="n">
+      <c r="D66" s="17" t="n">
         <f aca="false">MAX(B66-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -4066,24 +4286,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K66" s="18" t="n">
+      <c r="K66" s="21" t="n">
         <f aca="false">IF(I66&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="18" t="n">
+      <c r="A67" s="21" t="n">
         <v>7</v>
       </c>
-      <c r="B67" s="14" t="n">
+      <c r="B67" s="17" t="n">
         <f aca="false">A67*MES_HRS*WEEKS*(1+MES_DIM)^A67</f>
         <v>343.617898145328</v>
       </c>
-      <c r="C67" s="14" t="n">
+      <c r="C67" s="17" t="n">
         <f aca="false">MIN(B67,OWN_HRS)</f>
         <v>343.617898145328</v>
       </c>
-      <c r="D67" s="14" t="n">
+      <c r="D67" s="17" t="n">
         <f aca="false">MAX(B67-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -4111,24 +4331,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K67" s="18" t="n">
+      <c r="K67" s="21" t="n">
         <f aca="false">IF(I67&gt;=MES_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="18" t="n">
+      <c r="A68" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="B68" s="14" t="n">
+      <c r="B68" s="17" t="n">
         <f aca="false">A68*MES_HRS*WEEKS*(1+MES_DIM)^A68</f>
         <v>397.614996425308</v>
       </c>
-      <c r="C68" s="14" t="n">
+      <c r="C68" s="17" t="n">
         <f aca="false">MIN(B68,OWN_HRS)</f>
         <v>397.614996425308</v>
       </c>
-      <c r="D68" s="14" t="n">
+      <c r="D68" s="17" t="n">
         <f aca="false">MAX(B68-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -4156,24 +4376,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K68" s="18" t="n">
+      <c r="K68" s="21" t="n">
         <f aca="false">IF(I68&gt;=MES_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="18" t="n">
+      <c r="A69" s="21" t="n">
         <v>9</v>
       </c>
-      <c r="B69" s="14" t="n">
+      <c r="B69" s="17" t="n">
         <f aca="false">A69*MES_HRS*WEEKS*(1+MES_DIM)^A69</f>
         <v>452.908331865703</v>
       </c>
-      <c r="C69" s="14" t="n">
+      <c r="C69" s="17" t="n">
         <f aca="false">MIN(B69,OWN_HRS)</f>
         <v>452.908331865703</v>
       </c>
-      <c r="D69" s="14" t="n">
+      <c r="D69" s="17" t="n">
         <f aca="false">MAX(B69-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -4201,24 +4421,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K69" s="18" t="n">
+      <c r="K69" s="21" t="n">
         <f aca="false">IF(I69&gt;=MES_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="18" t="n">
+      <c r="A70" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="B70" s="14" t="n">
+      <c r="B70" s="17" t="n">
         <f aca="false">A70*MES_HRS*WEEKS*(1+MES_DIM)^A70</f>
         <v>509.521873348916</v>
       </c>
-      <c r="C70" s="14" t="n">
+      <c r="C70" s="17" t="n">
         <f aca="false">MIN(B70,OWN_HRS)</f>
         <v>509.521873348916</v>
       </c>
-      <c r="D70" s="14" t="n">
+      <c r="D70" s="17" t="n">
         <f aca="false">MAX(B70-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -4246,24 +4466,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K70" s="18" t="n">
+      <c r="K70" s="21" t="n">
         <f aca="false">IF(I70&gt;=MES_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="18" t="n">
+      <c r="A71" s="21" t="n">
         <v>11</v>
       </c>
-      <c r="B71" s="14" t="n">
+      <c r="B71" s="17" t="n">
         <f aca="false">A71*MES_HRS*WEEKS*(1+MES_DIM)^A71</f>
         <v>567.479986442355</v>
       </c>
-      <c r="C71" s="14" t="n">
+      <c r="C71" s="17" t="n">
         <f aca="false">MIN(B71,OWN_HRS)</f>
         <v>567.479986442355</v>
       </c>
-      <c r="D71" s="14" t="n">
+      <c r="D71" s="17" t="n">
         <f aca="false">MAX(B71-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -4291,24 +4511,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K71" s="18" t="n">
+      <c r="K71" s="21" t="n">
         <f aca="false">IF(I71&gt;=MES_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="18" t="n">
+      <c r="A72" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="B72" s="14" t="n">
+      <c r="B72" s="17" t="n">
         <f aca="false">A72*MES_HRS*WEEKS*(1+MES_DIM)^A72</f>
         <v>626.807439570419</v>
       </c>
-      <c r="C72" s="14" t="n">
+      <c r="C72" s="17" t="n">
         <f aca="false">MIN(B72,OWN_HRS)</f>
         <v>626.807439570419</v>
       </c>
-      <c r="D72" s="14" t="n">
+      <c r="D72" s="17" t="n">
         <f aca="false">MAX(B72-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -4336,24 +4556,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K72" s="18" t="n">
+      <c r="K72" s="21" t="n">
         <f aca="false">IF(I72&gt;=MES_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="18" t="n">
+      <c r="A73" s="21" t="n">
         <v>13</v>
       </c>
-      <c r="B73" s="14" t="n">
+      <c r="B73" s="17" t="n">
         <f aca="false">A73*MES_HRS*WEEKS*(1+MES_DIM)^A73</f>
         <v>687.529410278803</v>
       </c>
-      <c r="C73" s="14" t="n">
+      <c r="C73" s="17" t="n">
         <f aca="false">MIN(B73,OWN_HRS)</f>
         <v>687.529410278803</v>
       </c>
-      <c r="D73" s="14" t="n">
+      <c r="D73" s="17" t="n">
         <f aca="false">MAX(B73-OWN_HRS,0)</f>
         <v>0</v>
       </c>
@@ -4381,24 +4601,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K73" s="18" t="n">
+      <c r="K73" s="21" t="n">
         <f aca="false">IF(I73&gt;=MES_PRICE,1,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="18" t="n">
+      <c r="A74" s="21" t="n">
         <v>14</v>
       </c>
-      <c r="B74" s="14" t="n">
+      <c r="B74" s="17" t="n">
         <f aca="false">A74*MES_HRS*WEEKS*(1+MES_DIM)^A74</f>
         <v>749.671491592464</v>
       </c>
-      <c r="C74" s="14" t="n">
+      <c r="C74" s="17" t="n">
         <f aca="false">MIN(B74,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D74" s="14" t="n">
+      <c r="D74" s="17" t="n">
         <f aca="false">MAX(B74-OWN_HRS,0)</f>
         <v>29.6714915924644</v>
       </c>
@@ -4426,24 +4646,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K74" s="18" t="n">
+      <c r="K74" s="21" t="n">
         <f aca="false">IF(I74&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="18" t="n">
+      <c r="A75" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="B75" s="14" t="n">
+      <c r="B75" s="17" t="n">
         <f aca="false">A75*MES_HRS*WEEKS*(1+MES_DIM)^A75</f>
         <v>813.259698468611</v>
       </c>
-      <c r="C75" s="14" t="n">
+      <c r="C75" s="17" t="n">
         <f aca="false">MIN(B75,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D75" s="14" t="n">
+      <c r="D75" s="17" t="n">
         <f aca="false">MAX(B75-OWN_HRS,0)</f>
         <v>93.2596984686107</v>
       </c>
@@ -4471,24 +4691,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K75" s="18" t="n">
+      <c r="K75" s="21" t="n">
         <f aca="false">IF(I75&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="18" t="n">
+      <c r="A76" s="21" t="n">
         <v>16</v>
       </c>
-      <c r="B76" s="14" t="n">
+      <c r="B76" s="17" t="n">
         <f aca="false">A76*MES_HRS*WEEKS*(1+MES_DIM)^A76</f>
         <v>878.3204743461</v>
       </c>
-      <c r="C76" s="14" t="n">
+      <c r="C76" s="17" t="n">
         <f aca="false">MIN(B76,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D76" s="14" t="n">
+      <c r="D76" s="17" t="n">
         <f aca="false">MAX(B76-OWN_HRS,0)</f>
         <v>158.3204743461</v>
       </c>
@@ -4516,24 +4736,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K76" s="18" t="n">
+      <c r="K76" s="21" t="n">
         <f aca="false">IF(I76&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="18" t="n">
+      <c r="A77" s="21" t="n">
         <v>17</v>
       </c>
-      <c r="B77" s="14" t="n">
+      <c r="B77" s="17" t="n">
         <f aca="false">A77*MES_HRS*WEEKS*(1+MES_DIM)^A77</f>
         <v>944.88069779264</v>
       </c>
-      <c r="C77" s="14" t="n">
+      <c r="C77" s="17" t="n">
         <f aca="false">MIN(B77,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D77" s="14" t="n">
+      <c r="D77" s="17" t="n">
         <f aca="false">MAX(B77-OWN_HRS,0)</f>
         <v>224.88069779264</v>
       </c>
@@ -4561,24 +4781,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K77" s="18" t="n">
+      <c r="K77" s="21" t="n">
         <f aca="false">IF(I77&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="18" t="n">
+      <c r="A78" s="21" t="n">
         <v>18</v>
       </c>
-      <c r="B78" s="14" t="n">
+      <c r="B78" s="17" t="n">
         <f aca="false">A78*MES_HRS*WEEKS*(1+MES_DIM)^A78</f>
         <v>1012.96768925123</v>
       </c>
-      <c r="C78" s="14" t="n">
+      <c r="C78" s="17" t="n">
         <f aca="false">MIN(B78,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D78" s="14" t="n">
+      <c r="D78" s="17" t="n">
         <f aca="false">MAX(B78-OWN_HRS,0)</f>
         <v>292.967689251227</v>
       </c>
@@ -4606,24 +4826,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K78" s="18" t="n">
+      <c r="K78" s="21" t="n">
         <f aca="false">IF(I78&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="18" t="n">
+      <c r="A79" s="21" t="n">
         <v>19</v>
       </c>
-      <c r="B79" s="14" t="n">
+      <c r="B79" s="17" t="n">
         <f aca="false">A79*MES_HRS*WEEKS*(1+MES_DIM)^A79</f>
         <v>1082.60921788725</v>
       </c>
-      <c r="C79" s="14" t="n">
+      <c r="C79" s="17" t="n">
         <f aca="false">MIN(B79,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D79" s="14" t="n">
+      <c r="D79" s="17" t="n">
         <f aca="false">MAX(B79-OWN_HRS,0)</f>
         <v>362.609217887249</v>
       </c>
@@ -4651,24 +4871,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K79" s="18" t="n">
+      <c r="K79" s="21" t="n">
         <f aca="false">IF(I79&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="18" t="n">
+      <c r="A80" s="21" t="n">
         <v>20</v>
       </c>
-      <c r="B80" s="14" t="n">
+      <c r="B80" s="17" t="n">
         <f aca="false">A80*MES_HRS*WEEKS*(1+MES_DIM)^A80</f>
         <v>1153.83350853773</v>
       </c>
-      <c r="C80" s="14" t="n">
+      <c r="C80" s="17" t="n">
         <f aca="false">MIN(B80,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D80" s="14" t="n">
+      <c r="D80" s="17" t="n">
         <f aca="false">MAX(B80-OWN_HRS,0)</f>
         <v>433.833508537726</v>
       </c>
@@ -4696,24 +4916,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K80" s="18" t="n">
+      <c r="K80" s="21" t="n">
         <f aca="false">IF(I80&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="18" t="n">
+      <c r="A81" s="21" t="n">
         <v>21</v>
       </c>
-      <c r="B81" s="14" t="n">
+      <c r="B81" s="17" t="n">
         <f aca="false">A81*MES_HRS*WEEKS*(1+MES_DIM)^A81</f>
         <v>1226.66924876417</v>
       </c>
-      <c r="C81" s="14" t="n">
+      <c r="C81" s="17" t="n">
         <f aca="false">MIN(B81,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D81" s="14" t="n">
+      <c r="D81" s="17" t="n">
         <f aca="false">MAX(B81-OWN_HRS,0)</f>
         <v>506.66924876417</v>
       </c>
@@ -4741,24 +4961,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K81" s="18" t="n">
+      <c r="K81" s="21" t="n">
         <f aca="false">IF(I81&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="18" t="n">
+      <c r="A82" s="21" t="n">
         <v>22</v>
       </c>
-      <c r="B82" s="14" t="n">
+      <c r="B82" s="17" t="n">
         <f aca="false">A82*MES_HRS*WEEKS*(1+MES_DIM)^A82</f>
         <v>1301.14559601057</v>
       </c>
-      <c r="C82" s="14" t="n">
+      <c r="C82" s="17" t="n">
         <f aca="false">MIN(B82,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D82" s="14" t="n">
+      <c r="D82" s="17" t="n">
         <f aca="false">MAX(B82-OWN_HRS,0)</f>
         <v>581.145596010566</v>
       </c>
@@ -4786,24 +5006,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K82" s="18" t="n">
+      <c r="K82" s="21" t="n">
         <f aca="false">IF(I82&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="18" t="n">
+      <c r="A83" s="21" t="n">
         <v>23</v>
       </c>
-      <c r="B83" s="14" t="n">
+      <c r="B83" s="17" t="n">
         <f aca="false">A83*MES_HRS*WEEKS*(1+MES_DIM)^A83</f>
         <v>1377.292184868</v>
       </c>
-      <c r="C83" s="14" t="n">
+      <c r="C83" s="17" t="n">
         <f aca="false">MIN(B83,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D83" s="14" t="n">
+      <c r="D83" s="17" t="n">
         <f aca="false">MAX(B83-OWN_HRS,0)</f>
         <v>657.292184868002</v>
       </c>
@@ -4831,24 +5051,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K83" s="18" t="n">
+      <c r="K83" s="21" t="n">
         <f aca="false">IF(I83&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="18" t="n">
+      <c r="A84" s="21" t="n">
         <v>24</v>
       </c>
-      <c r="B84" s="14" t="n">
+      <c r="B84" s="17" t="n">
         <f aca="false">A84*MES_HRS*WEEKS*(1+MES_DIM)^A84</f>
         <v>1455.1391344475</v>
       </c>
-      <c r="C84" s="14" t="n">
+      <c r="C84" s="17" t="n">
         <f aca="false">MIN(B84,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D84" s="14" t="n">
+      <c r="D84" s="17" t="n">
         <f aca="false">MAX(B84-OWN_HRS,0)</f>
         <v>735.139134447498</v>
       </c>
@@ -4876,24 +5096,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K84" s="18" t="n">
+      <c r="K84" s="21" t="n">
         <f aca="false">IF(I84&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="18" t="n">
+      <c r="A85" s="21" t="n">
         <v>25</v>
       </c>
-      <c r="B85" s="14" t="n">
+      <c r="B85" s="17" t="n">
         <f aca="false">A85*MES_HRS*WEEKS*(1+MES_DIM)^A85</f>
         <v>1534.7170558626</v>
       </c>
-      <c r="C85" s="14" t="n">
+      <c r="C85" s="17" t="n">
         <f aca="false">MIN(B85,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D85" s="14" t="n">
+      <c r="D85" s="17" t="n">
         <f aca="false">MAX(B85-OWN_HRS,0)</f>
         <v>814.717055862596</v>
       </c>
@@ -4921,24 +5141,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K85" s="18" t="n">
+      <c r="K85" s="21" t="n">
         <f aca="false">IF(I85&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="18" t="n">
+      <c r="A86" s="21" t="n">
         <v>26</v>
       </c>
-      <c r="B86" s="14" t="n">
+      <c r="B86" s="17" t="n">
         <f aca="false">A86*MES_HRS*WEEKS*(1+MES_DIM)^A86</f>
         <v>1616.05705982331</v>
       </c>
-      <c r="C86" s="14" t="n">
+      <c r="C86" s="17" t="n">
         <f aca="false">MIN(B86,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D86" s="14" t="n">
+      <c r="D86" s="17" t="n">
         <f aca="false">MAX(B86-OWN_HRS,0)</f>
         <v>896.057059823313</v>
       </c>
@@ -4966,24 +5186,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K86" s="18" t="n">
+      <c r="K86" s="21" t="n">
         <f aca="false">IF(I86&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="18" t="n">
+      <c r="A87" s="21" t="n">
         <v>27</v>
       </c>
-      <c r="B87" s="14" t="n">
+      <c r="B87" s="17" t="n">
         <f aca="false">A87*MES_HRS*WEEKS*(1+MES_DIM)^A87</f>
         <v>1699.19076434307</v>
       </c>
-      <c r="C87" s="14" t="n">
+      <c r="C87" s="17" t="n">
         <f aca="false">MIN(B87,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D87" s="14" t="n">
+      <c r="D87" s="17" t="n">
         <f aca="false">MAX(B87-OWN_HRS,0)</f>
         <v>979.19076434307</v>
       </c>
@@ -5011,24 +5231,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K87" s="18" t="n">
+      <c r="K87" s="21" t="n">
         <f aca="false">IF(I87&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="18" t="n">
+      <c r="A88" s="21" t="n">
         <v>28</v>
       </c>
-      <c r="B88" s="14" t="n">
+      <c r="B88" s="17" t="n">
         <f aca="false">A88*MES_HRS*WEEKS*(1+MES_DIM)^A88</f>
         <v>1784.15030256022</v>
       </c>
-      <c r="C88" s="14" t="n">
+      <c r="C88" s="17" t="n">
         <f aca="false">MIN(B88,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D88" s="14" t="n">
+      <c r="D88" s="17" t="n">
         <f aca="false">MAX(B88-OWN_HRS,0)</f>
         <v>1064.15030256022</v>
       </c>
@@ -5056,24 +5276,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K88" s="18" t="n">
+      <c r="K88" s="21" t="n">
         <f aca="false">IF(I88&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="18" t="n">
+      <c r="A89" s="21" t="n">
         <v>29</v>
       </c>
-      <c r="B89" s="14" t="n">
+      <c r="B89" s="17" t="n">
         <f aca="false">A89*MES_HRS*WEEKS*(1+MES_DIM)^A89</f>
         <v>1870.96833067588</v>
       </c>
-      <c r="C89" s="14" t="n">
+      <c r="C89" s="17" t="n">
         <f aca="false">MIN(B89,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D89" s="14" t="n">
+      <c r="D89" s="17" t="n">
         <f aca="false">MAX(B89-OWN_HRS,0)</f>
         <v>1150.96833067588</v>
       </c>
@@ -5101,24 +5321,24 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K89" s="18" t="n">
+      <c r="K89" s="21" t="n">
         <f aca="false">IF(I89&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="18" t="n">
+      <c r="A90" s="21" t="n">
         <v>30</v>
       </c>
-      <c r="B90" s="14" t="n">
+      <c r="B90" s="17" t="n">
         <f aca="false">A90*MES_HRS*WEEKS*(1+MES_DIM)^A90</f>
         <v>1959.67803600965</v>
       </c>
-      <c r="C90" s="14" t="n">
+      <c r="C90" s="17" t="n">
         <f aca="false">MIN(B90,OWN_HRS)</f>
         <v>720</v>
       </c>
-      <c r="D90" s="14" t="n">
+      <c r="D90" s="17" t="n">
         <f aca="false">MAX(B90-OWN_HRS,0)</f>
         <v>1239.67803600965</v>
       </c>
@@ -5146,16 +5366,16 @@
         <f aca="false">MES_PRICE</f>
         <v>2700</v>
       </c>
-      <c r="K90" s="18" t="n">
+      <c r="K90" s="21" t="n">
         <f aca="false">IF(I90&gt;=MES_PRICE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="B92" s="19" t="n">
+        <v>102</v>
+      </c>
+      <c r="B92" s="22" t="n">
         <f aca="false">IF(ISNA(MATCH(1,'Marginal Cost Schedules'!$K$61:$K$90,0)),MES_CAP,MATCH(1,'Marginal Cost Schedules'!$K$61:$K$90,0)-1)</f>
         <v>6</v>
       </c>
@@ -5177,7 +5397,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D52"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="16"/>
@@ -5185,31 +5405,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="16" t="s">
-        <v>97</v>
+      <c r="A2" s="19" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="B5" s="14" t="n">
+        <v>106</v>
+      </c>
+      <c r="B5" s="17" t="n">
         <f aca="false">1*TOM_HRS*WEEKS*(1+TOM_DIM)^1</f>
         <v>99</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="B6" s="7" t="n">
         <v>99</v>
@@ -5217,21 +5437,21 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="B7" s="20" t="b">
+        <v>108</v>
+      </c>
+      <c r="B7" s="23" t="b">
         <f aca="false">B5=B6</f>
         <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="B10" s="11" t="n">
         <f aca="false">INDEX(MC_TOM,10)</f>
@@ -5240,331 +5460,349 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="B11" s="21"/>
+        <v>111</v>
+      </c>
+      <c r="B11" s="24" t="n">
+        <v>8249</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="B12" s="11" t="n">
         <f aca="false">ABS(B10-B11)</f>
-        <v>8248.1149448368</v>
+        <v>0.885055163198558</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="B13" s="20" t="b">
+        <v>113</v>
+      </c>
+      <c r="B13" s="23" t="b">
         <f aca="false">B12&lt;=1</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="2" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
+        <v>117</v>
+      </c>
+      <c r="B17" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
+        <v>118</v>
+      </c>
+      <c r="B18" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
+        <v>119</v>
+      </c>
+      <c r="B19" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="C19" s="10" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="B20" s="21"/>
-      <c r="C20" s="21"/>
+        <v>120</v>
+      </c>
+      <c r="B20" s="24" t="n">
+        <v>42775.17</v>
+      </c>
+      <c r="C20" s="24" t="n">
+        <v>42775.17</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="B21" s="20" t="b">
+        <v>121</v>
+      </c>
+      <c r="B21" s="23" t="b">
         <f aca="false">AND(B17=C17,B18=C18,B19=C19)</f>
         <v>1</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="B22" s="20" t="b">
+        <v>122</v>
+      </c>
+      <c r="B22" s="23" t="b">
         <f aca="false">ABS(B20-C20)&lt;=0.01</f>
         <v>1</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="2" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B26" s="18" t="n">
+        <v>126</v>
+      </c>
+      <c r="B26" s="21" t="n">
         <f aca="false">TOM_BEDS</f>
-        <v>0</v>
-      </c>
-      <c r="C26" s="18" t="n">
+        <v>10.004470073479</v>
+      </c>
+      <c r="C26" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="D26" s="20" t="b">
+      <c r="D26" s="23" t="b">
         <f aca="false">B26=C26</f>
         <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="B27" s="18" t="n">
+        <v>127</v>
+      </c>
+      <c r="B27" s="21" t="n">
         <f aca="false">CAR_BEDS</f>
-        <v>0</v>
-      </c>
-      <c r="C27" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="D27" s="20" t="b">
+      <c r="C27" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="D27" s="23" t="b">
         <f aca="false">B27=C27</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="B28" s="18" t="n">
+        <v>128</v>
+      </c>
+      <c r="B28" s="21" t="n">
         <f aca="false">MES_BEDS</f>
-        <v>0</v>
-      </c>
-      <c r="C28" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="D28" s="20" t="b">
+      <c r="C28" s="21" t="n">
+        <v>30</v>
+      </c>
+      <c r="D28" s="23" t="b">
         <f aca="false">B28=C28</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="B29" s="11" t="n">
         <f aca="false">PROFIT</f>
-        <v>-20000</v>
+        <v>42775.1669071729</v>
       </c>
       <c r="C29" s="11" t="n">
         <v>42762</v>
       </c>
-      <c r="D29" s="20" t="b">
+      <c r="D29" s="23" t="b">
         <f aca="false">ABS(B29-C29)&lt;=0.01</f>
         <v>0</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="B30" s="18" t="n">
+        <v>130</v>
+      </c>
+      <c r="B30" s="21" t="n">
         <f aca="false">TOM_CROSSING</f>
         <v>10</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="B31" s="18" t="n">
+        <v>132</v>
+      </c>
+      <c r="B31" s="21" t="n">
         <f aca="false">CAR_CROSSING</f>
         <v>10</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="B32" s="18" t="n">
+        <v>133</v>
+      </c>
+      <c r="B32" s="21" t="n">
         <f aca="false">MES_CROSSING</f>
         <v>6</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="9" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="9" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="B42" s="20" t="b">
+        <v>141</v>
+      </c>
+      <c r="B42" s="23" t="b">
         <f aca="false">TOM_BEDS&lt;=TOM_CAP</f>
         <v>1</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="B43" s="20" t="b">
+        <v>142</v>
+      </c>
+      <c r="B43" s="23" t="b">
         <f aca="false">CAR_BEDS&lt;=CAR_CAP</f>
         <v>1</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="B44" s="20" t="b">
+        <v>143</v>
+      </c>
+      <c r="B44" s="23" t="b">
         <f aca="false">MES_BEDS&lt;=MES_CAP</f>
         <v>1</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="B45" s="20" t="b">
+        <v>144</v>
+      </c>
+      <c r="B45" s="23" t="b">
         <f aca="false">(TOM_BEDS+CAR_BEDS+MES_BEDS)&lt;=TOTAL_BEDS</f>
         <v>1</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="B46" s="20" t="b">
+        <v>145</v>
+      </c>
+      <c r="B46" s="23" t="b">
         <f aca="false">TEMP_HRS_USED&lt;=(MAX_WORKERS*WORKER_HRS)</f>
         <v>1</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="B47" s="20" t="b">
+        <v>146</v>
+      </c>
+      <c r="B47" s="23" t="b">
         <f aca="false">TOM_BEDS&gt;=0</f>
         <v>1</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="B48" s="20" t="b">
+        <v>147</v>
+      </c>
+      <c r="B48" s="23" t="b">
         <f aca="false">CAR_BEDS&gt;=0</f>
         <v>1</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="B49" s="20" t="b">
+        <v>148</v>
+      </c>
+      <c r="B49" s="23" t="b">
         <f aca="false">MES_BEDS&gt;=0</f>
         <v>1</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="B50" s="20" t="b">
+        <v>149</v>
+      </c>
+      <c r="B50" s="23" t="b">
         <f aca="false">TOM_BEDS=ROUND(TOM_BEDS,0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="B51" s="20" t="b">
+        <v>150</v>
+      </c>
+      <c r="B51" s="23" t="b">
         <f aca="false">CAR_BEDS=ROUND(CAR_BEDS,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="B52" s="20" t="b">
+        <v>151</v>
+      </c>
+      <c r="B52" s="23" t="b">
         <f aca="false">MES_BEDS=ROUND(MES_BEDS,0)</f>
         <v>1</v>
       </c>
@@ -5579,146 +5817,34 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13">
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B21">
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+  <conditionalFormatting sqref="B21:B22">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B22">
-    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+  <conditionalFormatting sqref="D26:D29">
+    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D26">
-    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+  <conditionalFormatting sqref="B42:B52">
+    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D27">
-    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="13" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D28">
-    <cfRule type="cellIs" priority="14" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="15" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D29">
-    <cfRule type="cellIs" priority="16" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="17" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B42">
-    <cfRule type="cellIs" priority="18" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="19" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B43">
-    <cfRule type="cellIs" priority="20" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="21" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B44">
-    <cfRule type="cellIs" priority="22" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="23" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B45">
-    <cfRule type="cellIs" priority="24" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="25" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B46">
-    <cfRule type="cellIs" priority="26" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="27" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B47">
-    <cfRule type="cellIs" priority="28" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="29" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B48">
-    <cfRule type="cellIs" priority="30" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="31" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B49">
-    <cfRule type="cellIs" priority="32" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="33" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B50">
-    <cfRule type="cellIs" priority="34" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="35" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B51">
-    <cfRule type="cellIs" priority="36" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="37" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B52">
-    <cfRule type="cellIs" priority="38" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>1</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="39" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>